<commit_message>
feat(s3-2): implement any strategy, tactic and fundraiser features
</commit_message>
<xml_diff>
--- a/reports/Planning-Template.xlsx
+++ b/reports/Planning-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Manuel Zoilo\Documents\Universidad\DP2\DP2 - 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lcman\Desktop\DP2\Workspace-26\Projects\DP2-2526-G010\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5EF61CE-CD62-447F-9A08-404800219149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D422DDEB-0F7D-4850-8A2C-0114593C2DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="0" windowWidth="12960" windowHeight="13760" activeTab="3" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Copyright" sheetId="10" r:id="rId1"/>
@@ -48,6 +48,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -818,14 +821,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1471,12 +1474,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0BB59C7-21D2-4063-B60E-B9743CBEBCDD}">
   <dimension ref="B2:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1171875" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="9.1171875" style="1"/>
+    <col min="1" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="55" t="s">
         <v>94</v>
       </c>
@@ -1489,7 +1492,7 @@
       <c r="I2" s="55"/>
       <c r="J2" s="55"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B4" s="53" t="s">
         <v>3</v>
       </c>
@@ -1502,7 +1505,7 @@
       <c r="I4" s="54"/>
       <c r="J4" s="54"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="54"/>
       <c r="C5" s="54"/>
       <c r="D5" s="54"/>
@@ -1513,7 +1516,7 @@
       <c r="I5" s="54"/>
       <c r="J5" s="54"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="54"/>
       <c r="C6" s="54"/>
       <c r="D6" s="54"/>
@@ -1524,7 +1527,7 @@
       <c r="I6" s="54"/>
       <c r="J6" s="54"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="54"/>
       <c r="C7" s="54"/>
       <c r="D7" s="54"/>
@@ -1535,7 +1538,7 @@
       <c r="I7" s="54"/>
       <c r="J7" s="54"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="54"/>
       <c r="C8" s="54"/>
       <c r="D8" s="54"/>
@@ -1546,7 +1549,7 @@
       <c r="I8" s="54"/>
       <c r="J8" s="54"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="54"/>
       <c r="C9" s="54"/>
       <c r="D9" s="54"/>
@@ -1557,7 +1560,7 @@
       <c r="I9" s="54"/>
       <c r="J9" s="54"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B10" s="54"/>
       <c r="C10" s="54"/>
       <c r="D10" s="54"/>
@@ -1568,7 +1571,7 @@
       <c r="I10" s="54"/>
       <c r="J10" s="54"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B11" s="54"/>
       <c r="C11" s="54"/>
       <c r="D11" s="54"/>
@@ -1579,7 +1582,7 @@
       <c r="I11" s="54"/>
       <c r="J11" s="54"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B12" s="54"/>
       <c r="C12" s="54"/>
       <c r="D12" s="54"/>
@@ -1603,9 +1606,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BB35E99-EEE5-419C-812A-054E20454F46}">
   <dimension ref="B2:J13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="55" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1621,7 @@
       <c r="I2" s="55"/>
       <c r="J2" s="55"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1629,7 +1632,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="53" t="s">
         <v>4</v>
       </c>
@@ -1642,7 +1645,7 @@
       <c r="I4" s="53"/>
       <c r="J4" s="53"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="53"/>
       <c r="C5" s="53"/>
       <c r="D5" s="53"/>
@@ -1653,7 +1656,7 @@
       <c r="I5" s="53"/>
       <c r="J5" s="53"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="53"/>
       <c r="C6" s="53"/>
       <c r="D6" s="53"/>
@@ -1664,7 +1667,7 @@
       <c r="I6" s="53"/>
       <c r="J6" s="53"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1675,7 +1678,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="42"/>
       <c r="C8" s="43" t="s">
         <v>95</v>
@@ -1688,7 +1691,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="5"/>
       <c r="C9" s="56" t="s">
         <v>0</v>
@@ -1701,7 +1704,7 @@
       <c r="I9" s="56"/>
       <c r="J9" s="56"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B10" s="44"/>
       <c r="C10" s="56" t="s">
         <v>96</v>
@@ -1714,7 +1717,7 @@
       <c r="I10" s="56"/>
       <c r="J10" s="56"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B11" s="45"/>
       <c r="C11" s="56" t="s">
         <v>97</v>
@@ -1727,7 +1730,7 @@
       <c r="I11" s="56"/>
       <c r="J11" s="56"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
       <c r="C12" s="56" t="s">
         <v>2</v>
@@ -1740,7 +1743,7 @@
       <c r="I12" s="56"/>
       <c r="J12" s="56"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B13" s="4"/>
       <c r="C13" s="56" t="s">
         <v>1</v>
@@ -1770,13 +1773,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BAC9C64-283E-4A0D-9DEB-CD08499B2963}">
   <dimension ref="B2:J30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="1.703125" customWidth="1"/>
-    <col min="8" max="8" width="1.5859375" customWidth="1"/>
+    <col min="4" max="4" width="1.6640625" customWidth="1"/>
+    <col min="8" max="8" width="1.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="55" t="s">
         <v>5</v>
       </c>
@@ -1789,7 +1792,7 @@
       <c r="I2" s="55"/>
       <c r="J2" s="55"/>
     </row>
-    <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="53" t="s">
         <v>93</v>
       </c>
@@ -1802,7 +1805,7 @@
       <c r="I4" s="53"/>
       <c r="J4" s="53"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="53"/>
       <c r="C5" s="53"/>
       <c r="D5" s="53"/>
@@ -1813,7 +1816,7 @@
       <c r="I5" s="53"/>
       <c r="J5" s="53"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="53"/>
       <c r="C6" s="53"/>
       <c r="D6" s="53"/>
@@ -1824,7 +1827,7 @@
       <c r="I6" s="53"/>
       <c r="J6" s="53"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="53"/>
       <c r="C7" s="53"/>
       <c r="D7" s="53"/>
@@ -1835,7 +1838,7 @@
       <c r="I7" s="53"/>
       <c r="J7" s="53"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="37"/>
       <c r="C8" s="37"/>
       <c r="D8" s="37"/>
@@ -1846,11 +1849,11 @@
       <c r="I8" s="37"/>
       <c r="J8" s="37"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B10" s="57" t="s">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B10" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="57"/>
+      <c r="C10" s="59"/>
       <c r="E10" s="58" t="s">
         <v>98</v>
       </c>
@@ -1860,17 +1863,17 @@
       <c r="I10" s="58"/>
       <c r="J10" s="58"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B12" s="57" t="s">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B12" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="57"/>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B13" s="57" t="s">
+      <c r="C12" s="59"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B13" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="57"/>
+      <c r="C13" s="59"/>
       <c r="E13" s="58" t="s">
         <v>99</v>
       </c>
@@ -1884,15 +1887,15 @@
       </c>
       <c r="J13" s="58"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B14" s="57" t="s">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B14" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="57"/>
-      <c r="E14" s="59" t="s">
+      <c r="C14" s="59"/>
+      <c r="E14" s="57" t="s">
         <v>101</v>
       </c>
-      <c r="F14" s="59"/>
+      <c r="F14" s="57"/>
       <c r="G14" s="60" t="s">
         <v>17</v>
       </c>
@@ -1900,17 +1903,17 @@
       <c r="I14" s="61"/>
       <c r="J14" s="61"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B16" s="57" t="s">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B16" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="57"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B17" s="57" t="s">
+      <c r="C16" s="59"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B17" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="57"/>
+      <c r="C17" s="59"/>
       <c r="E17" s="58" t="s">
         <v>102</v>
       </c>
@@ -1924,15 +1927,15 @@
       </c>
       <c r="J17" s="58"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B18" s="57" t="s">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B18" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="E18" s="59" t="s">
+      <c r="C18" s="59"/>
+      <c r="E18" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="F18" s="59"/>
+      <c r="F18" s="57"/>
       <c r="G18" s="60" t="s">
         <v>17</v>
       </c>
@@ -1940,17 +1943,17 @@
       <c r="I18" s="61"/>
       <c r="J18" s="61"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B20" s="57" t="s">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B20" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="57"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B21" s="57" t="s">
+      <c r="C20" s="59"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B21" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="57"/>
+      <c r="C21" s="59"/>
       <c r="E21" s="58" t="s">
         <v>117</v>
       </c>
@@ -1964,15 +1967,15 @@
       </c>
       <c r="J21" s="58"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B22" s="57" t="s">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B22" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="57"/>
-      <c r="E22" s="59" t="s">
+      <c r="C22" s="59"/>
+      <c r="E22" s="57" t="s">
         <v>118</v>
       </c>
-      <c r="F22" s="59"/>
+      <c r="F22" s="57"/>
       <c r="G22" s="60" t="s">
         <v>17</v>
       </c>
@@ -1980,17 +1983,17 @@
       <c r="I22" s="61"/>
       <c r="J22" s="61"/>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B24" s="57" t="s">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B24" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="57"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B25" s="57" t="s">
+      <c r="C24" s="59"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B25" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="57"/>
+      <c r="C25" s="59"/>
       <c r="E25" s="58" t="s">
         <v>105</v>
       </c>
@@ -2004,15 +2007,15 @@
       </c>
       <c r="J25" s="58"/>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B26" s="57" t="s">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B26" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="57"/>
-      <c r="E26" s="59" t="s">
+      <c r="C26" s="59"/>
+      <c r="E26" s="57" t="s">
         <v>107</v>
       </c>
-      <c r="F26" s="59"/>
+      <c r="F26" s="57"/>
       <c r="G26" s="60" t="s">
         <v>17</v>
       </c>
@@ -2020,17 +2023,17 @@
       <c r="I26" s="61"/>
       <c r="J26" s="61"/>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B28" s="57" t="s">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B28" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="57"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B29" s="57" t="s">
+      <c r="C28" s="59"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B29" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="57"/>
+      <c r="C29" s="59"/>
       <c r="E29" s="58" t="s">
         <v>119</v>
       </c>
@@ -2044,15 +2047,15 @@
       </c>
       <c r="J29" s="58"/>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.5">
-      <c r="B30" s="57" t="s">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B30" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C30" s="57"/>
-      <c r="E30" s="59" t="s">
+      <c r="C30" s="59"/>
+      <c r="E30" s="57" t="s">
         <v>121</v>
       </c>
-      <c r="F30" s="59"/>
+      <c r="F30" s="57"/>
       <c r="G30" s="60" t="s">
         <v>17</v>
       </c>
@@ -2062,13 +2065,22 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E10:J10"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B4:J7"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="G14:J14"/>
@@ -2085,22 +2097,13 @@
     <mergeCell ref="I21:J21"/>
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="I25:J25"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E10:J10"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B4:J7"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E26:F26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2109,13 +2112,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34CF3CD5-8D08-494F-856F-AF84E30F468A}">
   <dimension ref="B2:P110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="15" width="18.87890625" customWidth="1"/>
-    <col min="16" max="16" width="64.5859375" customWidth="1"/>
+    <col min="3" max="15" width="18.88671875" customWidth="1"/>
+    <col min="16" max="16" width="64.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C2" s="55" t="s">
         <v>15</v>
       </c>
@@ -2133,7 +2136,7 @@
       <c r="O2" s="55"/>
       <c r="P2" s="55"/>
     </row>
-    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C4" s="53" t="s">
         <v>90</v>
       </c>
@@ -2151,7 +2154,7 @@
       <c r="O4" s="53"/>
       <c r="P4" s="53"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -2167,7 +2170,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C6" s="62" t="s">
         <v>83</v>
       </c>
@@ -2190,7 +2193,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C7" s="62"/>
       <c r="D7" s="13" t="s">
         <v>85</v>
@@ -2201,7 +2204,7 @@
       </c>
       <c r="J7" s="40"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -2224,7 +2227,7 @@
       <c r="O9" s="63"/>
       <c r="P9" s="9"/>
     </row>
-    <row r="10" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="10" t="s">
         <v>81</v>
       </c>
@@ -2271,7 +2274,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="46">
         <v>1</v>
       </c>
@@ -2318,7 +2321,7 @@
       </c>
       <c r="P11" s="49"/>
     </row>
-    <row r="12" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="46">
         <v>2</v>
       </c>
@@ -2366,7 +2369,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="46">
         <v>3</v>
       </c>
@@ -2414,7 +2417,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="46">
         <v>4</v>
       </c>
@@ -2438,7 +2441,9 @@
       <c r="I14" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="J14" s="51"/>
+      <c r="J14" s="51">
+        <v>46067.791666666664</v>
+      </c>
       <c r="K14" s="51">
         <v>46067.541666666664</v>
       </c>
@@ -2456,7 +2461,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="15" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="46">
         <v>5</v>
       </c>
@@ -2500,7 +2505,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="16" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="46">
         <v>6</v>
       </c>
@@ -2540,7 +2545,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="17" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="46">
         <v>7</v>
       </c>
@@ -2582,7 +2587,7 @@
       </c>
       <c r="P17" s="49"/>
     </row>
-    <row r="18" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="46">
         <v>8</v>
       </c>
@@ -2624,7 +2629,7 @@
       </c>
       <c r="P18" s="49"/>
     </row>
-    <row r="19" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="46">
         <v>9</v>
       </c>
@@ -2668,7 +2673,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="46">
         <v>10</v>
       </c>
@@ -2712,7 +2717,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="46">
         <v>11</v>
       </c>
@@ -2756,7 +2761,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="46">
         <v>12</v>
       </c>
@@ -2800,7 +2805,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="46">
         <v>13</v>
       </c>
@@ -2844,7 +2849,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="46">
         <v>14</v>
       </c>
@@ -2888,7 +2893,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="25" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="46">
         <v>15</v>
       </c>
@@ -2932,7 +2937,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="26" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="46">
         <v>16</v>
       </c>
@@ -2976,7 +2981,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="46">
         <v>17</v>
       </c>
@@ -3020,7 +3025,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="46">
         <v>18</v>
       </c>
@@ -3064,7 +3069,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="29" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="46">
         <v>19</v>
       </c>
@@ -3108,7 +3113,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="30" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="46">
         <v>20</v>
       </c>
@@ -3152,7 +3157,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="46">
         <v>21</v>
       </c>
@@ -3196,7 +3201,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="32" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="46">
         <v>22</v>
       </c>
@@ -3240,7 +3245,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="33" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="46">
         <v>23</v>
       </c>
@@ -3284,7 +3289,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="34" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="46">
         <v>24</v>
       </c>
@@ -3328,7 +3333,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="46">
         <v>25</v>
       </c>
@@ -3342,7 +3347,7 @@
       <c r="G35" s="48"/>
       <c r="H35" s="49"/>
       <c r="I35" s="50" t="str">
-        <f t="shared" ref="I30:I76" ca="1" si="0">IF(AND(J35="",K35=""),"",IF(AND(K35&lt;&gt;"",J35&gt;=NOW()),"Planned",IF(AND(K35&lt;&gt;"",K35&lt;NOW()),"Completed","Ongoing")))</f>
+        <f t="shared" ref="I35:I76" ca="1" si="0">IF(AND(J35="",K35=""),"",IF(AND(K35&lt;&gt;"",J35&gt;=NOW()),"Planned",IF(AND(K35&lt;&gt;"",K35&lt;NOW()),"Completed","Ongoing")))</f>
         <v/>
       </c>
       <c r="J35" s="51"/>
@@ -3359,7 +3364,7 @@
       </c>
       <c r="P35" s="49"/>
     </row>
-    <row r="36" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="46">
         <v>26</v>
       </c>
@@ -3390,7 +3395,7 @@
       </c>
       <c r="P36" s="49"/>
     </row>
-    <row r="37" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="46">
         <v>27</v>
       </c>
@@ -3421,7 +3426,7 @@
       </c>
       <c r="P37" s="49"/>
     </row>
-    <row r="38" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="46">
         <v>28</v>
       </c>
@@ -3452,7 +3457,7 @@
       </c>
       <c r="P38" s="49"/>
     </row>
-    <row r="39" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="46">
         <v>29</v>
       </c>
@@ -3483,7 +3488,7 @@
       </c>
       <c r="P39" s="49"/>
     </row>
-    <row r="40" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="46">
         <v>30</v>
       </c>
@@ -3514,7 +3519,7 @@
       </c>
       <c r="P40" s="49"/>
     </row>
-    <row r="41" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="46">
         <v>31</v>
       </c>
@@ -3545,7 +3550,7 @@
       </c>
       <c r="P41" s="49"/>
     </row>
-    <row r="42" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="46">
         <v>32</v>
       </c>
@@ -3576,7 +3581,7 @@
       </c>
       <c r="P42" s="49"/>
     </row>
-    <row r="43" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="46">
         <v>33</v>
       </c>
@@ -3607,7 +3612,7 @@
       </c>
       <c r="P43" s="49"/>
     </row>
-    <row r="44" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="46">
         <v>34</v>
       </c>
@@ -3638,7 +3643,7 @@
       </c>
       <c r="P44" s="49"/>
     </row>
-    <row r="45" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B45" s="46">
         <v>35</v>
       </c>
@@ -3669,7 +3674,7 @@
       </c>
       <c r="P45" s="49"/>
     </row>
-    <row r="46" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B46" s="46">
         <v>36</v>
       </c>
@@ -3700,7 +3705,7 @@
       </c>
       <c r="P46" s="49"/>
     </row>
-    <row r="47" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="46">
         <v>37</v>
       </c>
@@ -3731,7 +3736,7 @@
       </c>
       <c r="P47" s="49"/>
     </row>
-    <row r="48" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="46">
         <v>38</v>
       </c>
@@ -3762,7 +3767,7 @@
       </c>
       <c r="P48" s="49"/>
     </row>
-    <row r="49" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="46">
         <v>39</v>
       </c>
@@ -3793,7 +3798,7 @@
       </c>
       <c r="P49" s="49"/>
     </row>
-    <row r="50" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="46">
         <v>40</v>
       </c>
@@ -3824,7 +3829,7 @@
       </c>
       <c r="P50" s="49"/>
     </row>
-    <row r="51" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="46">
         <v>41</v>
       </c>
@@ -3855,7 +3860,7 @@
       </c>
       <c r="P51" s="49"/>
     </row>
-    <row r="52" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B52" s="46">
         <v>42</v>
       </c>
@@ -3886,7 +3891,7 @@
       </c>
       <c r="P52" s="49"/>
     </row>
-    <row r="53" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B53" s="46">
         <v>43</v>
       </c>
@@ -3917,7 +3922,7 @@
       </c>
       <c r="P53" s="49"/>
     </row>
-    <row r="54" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="46">
         <v>44</v>
       </c>
@@ -3948,7 +3953,7 @@
       </c>
       <c r="P54" s="49"/>
     </row>
-    <row r="55" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B55" s="46">
         <v>45</v>
       </c>
@@ -3979,7 +3984,7 @@
       </c>
       <c r="P55" s="49"/>
     </row>
-    <row r="56" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B56" s="46">
         <v>46</v>
       </c>
@@ -4010,7 +4015,7 @@
       </c>
       <c r="P56" s="49"/>
     </row>
-    <row r="57" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="46">
         <v>47</v>
       </c>
@@ -4041,7 +4046,7 @@
       </c>
       <c r="P57" s="49"/>
     </row>
-    <row r="58" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B58" s="46">
         <v>48</v>
       </c>
@@ -4072,7 +4077,7 @@
       </c>
       <c r="P58" s="49"/>
     </row>
-    <row r="59" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B59" s="46">
         <v>49</v>
       </c>
@@ -4103,7 +4108,7 @@
       </c>
       <c r="P59" s="49"/>
     </row>
-    <row r="60" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="46">
         <v>50</v>
       </c>
@@ -4134,7 +4139,7 @@
       </c>
       <c r="P60" s="49"/>
     </row>
-    <row r="61" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="46">
         <v>51</v>
       </c>
@@ -4165,7 +4170,7 @@
       </c>
       <c r="P61" s="49"/>
     </row>
-    <row r="62" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="46">
         <v>52</v>
       </c>
@@ -4196,7 +4201,7 @@
       </c>
       <c r="P62" s="49"/>
     </row>
-    <row r="63" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B63" s="46">
         <v>53</v>
       </c>
@@ -4227,7 +4232,7 @@
       </c>
       <c r="P63" s="49"/>
     </row>
-    <row r="64" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B64" s="46">
         <v>54</v>
       </c>
@@ -4258,7 +4263,7 @@
       </c>
       <c r="P64" s="49"/>
     </row>
-    <row r="65" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="46">
         <v>55</v>
       </c>
@@ -4289,7 +4294,7 @@
       </c>
       <c r="P65" s="49"/>
     </row>
-    <row r="66" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B66" s="46">
         <v>56</v>
       </c>
@@ -4320,7 +4325,7 @@
       </c>
       <c r="P66" s="49"/>
     </row>
-    <row r="67" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B67" s="46">
         <v>57</v>
       </c>
@@ -4351,7 +4356,7 @@
       </c>
       <c r="P67" s="49"/>
     </row>
-    <row r="68" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B68" s="46">
         <v>58</v>
       </c>
@@ -4382,7 +4387,7 @@
       </c>
       <c r="P68" s="49"/>
     </row>
-    <row r="69" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B69" s="46">
         <v>59</v>
       </c>
@@ -4413,7 +4418,7 @@
       </c>
       <c r="P69" s="49"/>
     </row>
-    <row r="70" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B70" s="46">
         <v>60</v>
       </c>
@@ -4444,7 +4449,7 @@
       </c>
       <c r="P70" s="49"/>
     </row>
-    <row r="71" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B71" s="46">
         <v>61</v>
       </c>
@@ -4475,7 +4480,7 @@
       </c>
       <c r="P71" s="49"/>
     </row>
-    <row r="72" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B72" s="46">
         <v>62</v>
       </c>
@@ -4506,7 +4511,7 @@
       </c>
       <c r="P72" s="49"/>
     </row>
-    <row r="73" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B73" s="46">
         <v>63</v>
       </c>
@@ -4537,7 +4542,7 @@
       </c>
       <c r="P73" s="49"/>
     </row>
-    <row r="74" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B74" s="46">
         <v>64</v>
       </c>
@@ -4568,7 +4573,7 @@
       </c>
       <c r="P74" s="49"/>
     </row>
-    <row r="75" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B75" s="46">
         <v>65</v>
       </c>
@@ -4599,7 +4604,7 @@
       </c>
       <c r="P75" s="49"/>
     </row>
-    <row r="76" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B76" s="46">
         <v>66</v>
       </c>
@@ -4630,7 +4635,7 @@
       </c>
       <c r="P76" s="49"/>
     </row>
-    <row r="77" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B77" s="46">
         <v>67</v>
       </c>
@@ -4661,7 +4666,7 @@
       </c>
       <c r="P77" s="49"/>
     </row>
-    <row r="78" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B78" s="46">
         <v>68</v>
       </c>
@@ -4692,7 +4697,7 @@
       </c>
       <c r="P78" s="49"/>
     </row>
-    <row r="79" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B79" s="46">
         <v>69</v>
       </c>
@@ -4723,7 +4728,7 @@
       </c>
       <c r="P79" s="49"/>
     </row>
-    <row r="80" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B80" s="46">
         <v>70</v>
       </c>
@@ -4754,7 +4759,7 @@
       </c>
       <c r="P80" s="49"/>
     </row>
-    <row r="81" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B81" s="46">
         <v>71</v>
       </c>
@@ -4785,7 +4790,7 @@
       </c>
       <c r="P81" s="49"/>
     </row>
-    <row r="82" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B82" s="46">
         <v>72</v>
       </c>
@@ -4816,7 +4821,7 @@
       </c>
       <c r="P82" s="49"/>
     </row>
-    <row r="83" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B83" s="46">
         <v>73</v>
       </c>
@@ -4847,7 +4852,7 @@
       </c>
       <c r="P83" s="49"/>
     </row>
-    <row r="84" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B84" s="46">
         <v>74</v>
       </c>
@@ -4878,7 +4883,7 @@
       </c>
       <c r="P84" s="49"/>
     </row>
-    <row r="85" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B85" s="46">
         <v>75</v>
       </c>
@@ -4909,7 +4914,7 @@
       </c>
       <c r="P85" s="49"/>
     </row>
-    <row r="86" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B86" s="46">
         <v>76</v>
       </c>
@@ -4940,7 +4945,7 @@
       </c>
       <c r="P86" s="49"/>
     </row>
-    <row r="87" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B87" s="46">
         <v>77</v>
       </c>
@@ -4971,7 +4976,7 @@
       </c>
       <c r="P87" s="49"/>
     </row>
-    <row r="88" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B88" s="46">
         <v>78</v>
       </c>
@@ -5002,7 +5007,7 @@
       </c>
       <c r="P88" s="49"/>
     </row>
-    <row r="89" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B89" s="46">
         <v>79</v>
       </c>
@@ -5033,7 +5038,7 @@
       </c>
       <c r="P89" s="49"/>
     </row>
-    <row r="90" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B90" s="46">
         <v>80</v>
       </c>
@@ -5064,7 +5069,7 @@
       </c>
       <c r="P90" s="49"/>
     </row>
-    <row r="91" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B91" s="46">
         <v>81</v>
       </c>
@@ -5095,7 +5100,7 @@
       </c>
       <c r="P91" s="49"/>
     </row>
-    <row r="92" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B92" s="46">
         <v>82</v>
       </c>
@@ -5126,7 +5131,7 @@
       </c>
       <c r="P92" s="49"/>
     </row>
-    <row r="93" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B93" s="46">
         <v>83</v>
       </c>
@@ -5157,7 +5162,7 @@
       </c>
       <c r="P93" s="49"/>
     </row>
-    <row r="94" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B94" s="46">
         <v>84</v>
       </c>
@@ -5188,7 +5193,7 @@
       </c>
       <c r="P94" s="49"/>
     </row>
-    <row r="95" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B95" s="46">
         <v>85</v>
       </c>
@@ -5219,7 +5224,7 @@
       </c>
       <c r="P95" s="49"/>
     </row>
-    <row r="96" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B96" s="46">
         <v>86</v>
       </c>
@@ -5250,7 +5255,7 @@
       </c>
       <c r="P96" s="49"/>
     </row>
-    <row r="97" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B97" s="46">
         <v>87</v>
       </c>
@@ -5281,7 +5286,7 @@
       </c>
       <c r="P97" s="49"/>
     </row>
-    <row r="98" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B98" s="46">
         <v>88</v>
       </c>
@@ -5312,7 +5317,7 @@
       </c>
       <c r="P98" s="49"/>
     </row>
-    <row r="99" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B99" s="46">
         <v>89</v>
       </c>
@@ -5343,7 +5348,7 @@
       </c>
       <c r="P99" s="49"/>
     </row>
-    <row r="100" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B100" s="46">
         <v>90</v>
       </c>
@@ -5374,7 +5379,7 @@
       </c>
       <c r="P100" s="49"/>
     </row>
-    <row r="101" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B101" s="46">
         <v>91</v>
       </c>
@@ -5405,7 +5410,7 @@
       </c>
       <c r="P101" s="49"/>
     </row>
-    <row r="102" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B102" s="46">
         <v>92</v>
       </c>
@@ -5436,7 +5441,7 @@
       </c>
       <c r="P102" s="49"/>
     </row>
-    <row r="103" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B103" s="46">
         <v>93</v>
       </c>
@@ -5467,7 +5472,7 @@
       </c>
       <c r="P103" s="49"/>
     </row>
-    <row r="104" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B104" s="46">
         <v>94</v>
       </c>
@@ -5498,7 +5503,7 @@
       </c>
       <c r="P104" s="49"/>
     </row>
-    <row r="105" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B105" s="46">
         <v>95</v>
       </c>
@@ -5529,7 +5534,7 @@
       </c>
       <c r="P105" s="49"/>
     </row>
-    <row r="106" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B106" s="46">
         <v>96</v>
       </c>
@@ -5560,7 +5565,7 @@
       </c>
       <c r="P106" s="49"/>
     </row>
-    <row r="107" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B107" s="46">
         <v>97</v>
       </c>
@@ -5591,7 +5596,7 @@
       </c>
       <c r="P107" s="49"/>
     </row>
-    <row r="108" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B108" s="46">
         <v>98</v>
       </c>
@@ -5622,7 +5627,7 @@
       </c>
       <c r="P108" s="49"/>
     </row>
-    <row r="109" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B109" s="46">
         <v>99</v>
       </c>
@@ -5653,7 +5658,7 @@
       </c>
       <c r="P109" s="49"/>
     </row>
-    <row r="110" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B110" s="46">
         <v>100</v>
       </c>
@@ -5704,7 +5709,7 @@
       <formula>$J$11&gt;$K$11</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="3343" yWindow="1045" count="10">
+  <dataValidations xWindow="1257" yWindow="712" count="10">
     <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Expected workload" prompt="Enter the expected workload in hours or fractions." sqref="L11:L110" xr:uid="{AADDA758-A288-4920-A868-A656B94EE475}">
       <formula1>0</formula1>
       <formula2>1024</formula2>
@@ -5727,7 +5732,7 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="3343" yWindow="1045" count="5">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1257" yWindow="712" count="5">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Role" prompt="Select a role from the select box.  Use &quot;other&quot; only in truly exceptional cases.  Consult your lecturer in such cases._x000a_" xr:uid="{A1102D1C-503C-44C5-9E57-51358D36832C}">
           <x14:formula1>
             <xm:f>Internal!$B$26:$B$32</xm:f>
@@ -5748,10 +5753,10 @@
         </x14:dataValidation>
         <x14:dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Start moment" prompt="Indicate the moment when the assignee starts working on this task.  Use format yy/mm/dd hh:mm." xr:uid="{3F118E98-586C-439A-BA73-E3236BC1E529}">
           <x14:formula1>
-            <xm:f>Internal!C22</xm:f>
+            <xm:f>Internal!B19</xm:f>
           </x14:formula1>
           <x14:formula2>
-            <xm:f>Internal!C23</xm:f>
+            <xm:f>Internal!B20</xm:f>
           </x14:formula2>
           <xm:sqref>J11:J110</xm:sqref>
         </x14:dataValidation>
@@ -5773,13 +5778,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28A4DB1-CB48-4778-AC73-C91746932E53}">
   <dimension ref="B2:P110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="15" width="18.87890625" customWidth="1"/>
-    <col min="16" max="16" width="64.5859375" customWidth="1"/>
+    <col min="3" max="15" width="18.88671875" customWidth="1"/>
+    <col min="16" max="16" width="64.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C2" s="55" t="s">
         <v>15</v>
       </c>
@@ -5797,7 +5802,7 @@
       <c r="O2" s="55"/>
       <c r="P2" s="55"/>
     </row>
-    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C4" s="53" t="s">
         <v>90</v>
       </c>
@@ -5815,7 +5820,7 @@
       <c r="O4" s="53"/>
       <c r="P4" s="53"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -5831,7 +5836,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C6" s="62" t="s">
         <v>83</v>
       </c>
@@ -5854,7 +5859,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C7" s="62"/>
       <c r="D7" s="13" t="s">
         <v>85</v>
@@ -5865,7 +5870,7 @@
       </c>
       <c r="J7" s="40"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -5888,7 +5893,7 @@
       <c r="O9" s="63"/>
       <c r="P9" s="9"/>
     </row>
-    <row r="10" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="10" t="s">
         <v>81</v>
       </c>
@@ -5935,7 +5940,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="46">
         <v>1</v>
       </c>
@@ -5966,7 +5971,7 @@
       </c>
       <c r="P11" s="49"/>
     </row>
-    <row r="12" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="46">
         <v>2</v>
       </c>
@@ -5997,7 +6002,7 @@
       </c>
       <c r="P12" s="49"/>
     </row>
-    <row r="13" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="46">
         <v>3</v>
       </c>
@@ -6028,7 +6033,7 @@
       </c>
       <c r="P13" s="49"/>
     </row>
-    <row r="14" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="46">
         <v>4</v>
       </c>
@@ -6059,7 +6064,7 @@
       </c>
       <c r="P14" s="49"/>
     </row>
-    <row r="15" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="46">
         <v>5</v>
       </c>
@@ -6090,7 +6095,7 @@
       </c>
       <c r="P15" s="49"/>
     </row>
-    <row r="16" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="46">
         <v>6</v>
       </c>
@@ -6121,7 +6126,7 @@
       </c>
       <c r="P16" s="49"/>
     </row>
-    <row r="17" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="46">
         <v>7</v>
       </c>
@@ -6152,7 +6157,7 @@
       </c>
       <c r="P17" s="49"/>
     </row>
-    <row r="18" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="46">
         <v>8</v>
       </c>
@@ -6183,7 +6188,7 @@
       </c>
       <c r="P18" s="49"/>
     </row>
-    <row r="19" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="46">
         <v>9</v>
       </c>
@@ -6214,7 +6219,7 @@
       </c>
       <c r="P19" s="49"/>
     </row>
-    <row r="20" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="46">
         <v>10</v>
       </c>
@@ -6245,7 +6250,7 @@
       </c>
       <c r="P20" s="49"/>
     </row>
-    <row r="21" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="46">
         <v>11</v>
       </c>
@@ -6276,7 +6281,7 @@
       </c>
       <c r="P21" s="49"/>
     </row>
-    <row r="22" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="46">
         <v>12</v>
       </c>
@@ -6307,7 +6312,7 @@
       </c>
       <c r="P22" s="49"/>
     </row>
-    <row r="23" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="46">
         <v>13</v>
       </c>
@@ -6338,7 +6343,7 @@
       </c>
       <c r="P23" s="49"/>
     </row>
-    <row r="24" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="46">
         <v>14</v>
       </c>
@@ -6369,7 +6374,7 @@
       </c>
       <c r="P24" s="49"/>
     </row>
-    <row r="25" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="46">
         <v>15</v>
       </c>
@@ -6400,7 +6405,7 @@
       </c>
       <c r="P25" s="49"/>
     </row>
-    <row r="26" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="46">
         <v>16</v>
       </c>
@@ -6431,7 +6436,7 @@
       </c>
       <c r="P26" s="49"/>
     </row>
-    <row r="27" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="46">
         <v>17</v>
       </c>
@@ -6462,7 +6467,7 @@
       </c>
       <c r="P27" s="49"/>
     </row>
-    <row r="28" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="46">
         <v>18</v>
       </c>
@@ -6493,7 +6498,7 @@
       </c>
       <c r="P28" s="49"/>
     </row>
-    <row r="29" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="46">
         <v>19</v>
       </c>
@@ -6524,7 +6529,7 @@
       </c>
       <c r="P29" s="49"/>
     </row>
-    <row r="30" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="46">
         <v>20</v>
       </c>
@@ -6555,7 +6560,7 @@
       </c>
       <c r="P30" s="49"/>
     </row>
-    <row r="31" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="46">
         <v>21</v>
       </c>
@@ -6586,7 +6591,7 @@
       </c>
       <c r="P31" s="49"/>
     </row>
-    <row r="32" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="46">
         <v>22</v>
       </c>
@@ -6617,7 +6622,7 @@
       </c>
       <c r="P32" s="49"/>
     </row>
-    <row r="33" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="46">
         <v>23</v>
       </c>
@@ -6648,7 +6653,7 @@
       </c>
       <c r="P33" s="49"/>
     </row>
-    <row r="34" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="46">
         <v>24</v>
       </c>
@@ -6679,7 +6684,7 @@
       </c>
       <c r="P34" s="49"/>
     </row>
-    <row r="35" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="46">
         <v>25</v>
       </c>
@@ -6710,7 +6715,7 @@
       </c>
       <c r="P35" s="49"/>
     </row>
-    <row r="36" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="46">
         <v>26</v>
       </c>
@@ -6741,7 +6746,7 @@
       </c>
       <c r="P36" s="49"/>
     </row>
-    <row r="37" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="46">
         <v>27</v>
       </c>
@@ -6772,7 +6777,7 @@
       </c>
       <c r="P37" s="49"/>
     </row>
-    <row r="38" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="46">
         <v>28</v>
       </c>
@@ -6803,7 +6808,7 @@
       </c>
       <c r="P38" s="49"/>
     </row>
-    <row r="39" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="46">
         <v>29</v>
       </c>
@@ -6834,7 +6839,7 @@
       </c>
       <c r="P39" s="49"/>
     </row>
-    <row r="40" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="46">
         <v>30</v>
       </c>
@@ -6865,7 +6870,7 @@
       </c>
       <c r="P40" s="49"/>
     </row>
-    <row r="41" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="46">
         <v>31</v>
       </c>
@@ -6896,7 +6901,7 @@
       </c>
       <c r="P41" s="49"/>
     </row>
-    <row r="42" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="46">
         <v>32</v>
       </c>
@@ -6927,7 +6932,7 @@
       </c>
       <c r="P42" s="49"/>
     </row>
-    <row r="43" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="46">
         <v>33</v>
       </c>
@@ -6958,7 +6963,7 @@
       </c>
       <c r="P43" s="49"/>
     </row>
-    <row r="44" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="46">
         <v>34</v>
       </c>
@@ -6989,7 +6994,7 @@
       </c>
       <c r="P44" s="49"/>
     </row>
-    <row r="45" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B45" s="46">
         <v>35</v>
       </c>
@@ -7020,7 +7025,7 @@
       </c>
       <c r="P45" s="49"/>
     </row>
-    <row r="46" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B46" s="46">
         <v>36</v>
       </c>
@@ -7051,7 +7056,7 @@
       </c>
       <c r="P46" s="49"/>
     </row>
-    <row r="47" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="46">
         <v>37</v>
       </c>
@@ -7082,7 +7087,7 @@
       </c>
       <c r="P47" s="49"/>
     </row>
-    <row r="48" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="46">
         <v>38</v>
       </c>
@@ -7113,7 +7118,7 @@
       </c>
       <c r="P48" s="49"/>
     </row>
-    <row r="49" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="46">
         <v>39</v>
       </c>
@@ -7144,7 +7149,7 @@
       </c>
       <c r="P49" s="49"/>
     </row>
-    <row r="50" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="46">
         <v>40</v>
       </c>
@@ -7175,7 +7180,7 @@
       </c>
       <c r="P50" s="49"/>
     </row>
-    <row r="51" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="46">
         <v>41</v>
       </c>
@@ -7206,7 +7211,7 @@
       </c>
       <c r="P51" s="49"/>
     </row>
-    <row r="52" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B52" s="46">
         <v>42</v>
       </c>
@@ -7237,7 +7242,7 @@
       </c>
       <c r="P52" s="49"/>
     </row>
-    <row r="53" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B53" s="46">
         <v>43</v>
       </c>
@@ -7268,7 +7273,7 @@
       </c>
       <c r="P53" s="49"/>
     </row>
-    <row r="54" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="46">
         <v>44</v>
       </c>
@@ -7299,7 +7304,7 @@
       </c>
       <c r="P54" s="49"/>
     </row>
-    <row r="55" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B55" s="46">
         <v>45</v>
       </c>
@@ -7330,7 +7335,7 @@
       </c>
       <c r="P55" s="49"/>
     </row>
-    <row r="56" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B56" s="46">
         <v>46</v>
       </c>
@@ -7361,7 +7366,7 @@
       </c>
       <c r="P56" s="49"/>
     </row>
-    <row r="57" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="46">
         <v>47</v>
       </c>
@@ -7392,7 +7397,7 @@
       </c>
       <c r="P57" s="49"/>
     </row>
-    <row r="58" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B58" s="46">
         <v>48</v>
       </c>
@@ -7423,7 +7428,7 @@
       </c>
       <c r="P58" s="49"/>
     </row>
-    <row r="59" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B59" s="46">
         <v>49</v>
       </c>
@@ -7454,7 +7459,7 @@
       </c>
       <c r="P59" s="49"/>
     </row>
-    <row r="60" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="46">
         <v>50</v>
       </c>
@@ -7485,7 +7490,7 @@
       </c>
       <c r="P60" s="49"/>
     </row>
-    <row r="61" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="46">
         <v>51</v>
       </c>
@@ -7516,7 +7521,7 @@
       </c>
       <c r="P61" s="49"/>
     </row>
-    <row r="62" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="46">
         <v>52</v>
       </c>
@@ -7547,7 +7552,7 @@
       </c>
       <c r="P62" s="49"/>
     </row>
-    <row r="63" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B63" s="46">
         <v>53</v>
       </c>
@@ -7578,7 +7583,7 @@
       </c>
       <c r="P63" s="49"/>
     </row>
-    <row r="64" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B64" s="46">
         <v>54</v>
       </c>
@@ -7609,7 +7614,7 @@
       </c>
       <c r="P64" s="49"/>
     </row>
-    <row r="65" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="46">
         <v>55</v>
       </c>
@@ -7640,7 +7645,7 @@
       </c>
       <c r="P65" s="49"/>
     </row>
-    <row r="66" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B66" s="46">
         <v>56</v>
       </c>
@@ -7671,7 +7676,7 @@
       </c>
       <c r="P66" s="49"/>
     </row>
-    <row r="67" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B67" s="46">
         <v>57</v>
       </c>
@@ -7702,7 +7707,7 @@
       </c>
       <c r="P67" s="49"/>
     </row>
-    <row r="68" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B68" s="46">
         <v>58</v>
       </c>
@@ -7733,7 +7738,7 @@
       </c>
       <c r="P68" s="49"/>
     </row>
-    <row r="69" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B69" s="46">
         <v>59</v>
       </c>
@@ -7764,7 +7769,7 @@
       </c>
       <c r="P69" s="49"/>
     </row>
-    <row r="70" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B70" s="46">
         <v>60</v>
       </c>
@@ -7795,7 +7800,7 @@
       </c>
       <c r="P70" s="49"/>
     </row>
-    <row r="71" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B71" s="46">
         <v>61</v>
       </c>
@@ -7826,7 +7831,7 @@
       </c>
       <c r="P71" s="49"/>
     </row>
-    <row r="72" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B72" s="46">
         <v>62</v>
       </c>
@@ -7857,7 +7862,7 @@
       </c>
       <c r="P72" s="49"/>
     </row>
-    <row r="73" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B73" s="46">
         <v>63</v>
       </c>
@@ -7888,7 +7893,7 @@
       </c>
       <c r="P73" s="49"/>
     </row>
-    <row r="74" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B74" s="46">
         <v>64</v>
       </c>
@@ -7919,7 +7924,7 @@
       </c>
       <c r="P74" s="49"/>
     </row>
-    <row r="75" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B75" s="46">
         <v>65</v>
       </c>
@@ -7950,7 +7955,7 @@
       </c>
       <c r="P75" s="49"/>
     </row>
-    <row r="76" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B76" s="46">
         <v>66</v>
       </c>
@@ -7981,7 +7986,7 @@
       </c>
       <c r="P76" s="49"/>
     </row>
-    <row r="77" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B77" s="46">
         <v>67</v>
       </c>
@@ -8012,7 +8017,7 @@
       </c>
       <c r="P77" s="49"/>
     </row>
-    <row r="78" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B78" s="46">
         <v>68</v>
       </c>
@@ -8043,7 +8048,7 @@
       </c>
       <c r="P78" s="49"/>
     </row>
-    <row r="79" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B79" s="46">
         <v>69</v>
       </c>
@@ -8074,7 +8079,7 @@
       </c>
       <c r="P79" s="49"/>
     </row>
-    <row r="80" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B80" s="46">
         <v>70</v>
       </c>
@@ -8105,7 +8110,7 @@
       </c>
       <c r="P80" s="49"/>
     </row>
-    <row r="81" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B81" s="46">
         <v>71</v>
       </c>
@@ -8136,7 +8141,7 @@
       </c>
       <c r="P81" s="49"/>
     </row>
-    <row r="82" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B82" s="46">
         <v>72</v>
       </c>
@@ -8167,7 +8172,7 @@
       </c>
       <c r="P82" s="49"/>
     </row>
-    <row r="83" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B83" s="46">
         <v>73</v>
       </c>
@@ -8198,7 +8203,7 @@
       </c>
       <c r="P83" s="49"/>
     </row>
-    <row r="84" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B84" s="46">
         <v>74</v>
       </c>
@@ -8229,7 +8234,7 @@
       </c>
       <c r="P84" s="49"/>
     </row>
-    <row r="85" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B85" s="46">
         <v>75</v>
       </c>
@@ -8260,7 +8265,7 @@
       </c>
       <c r="P85" s="49"/>
     </row>
-    <row r="86" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B86" s="46">
         <v>76</v>
       </c>
@@ -8291,7 +8296,7 @@
       </c>
       <c r="P86" s="49"/>
     </row>
-    <row r="87" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B87" s="46">
         <v>77</v>
       </c>
@@ -8322,7 +8327,7 @@
       </c>
       <c r="P87" s="49"/>
     </row>
-    <row r="88" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B88" s="46">
         <v>78</v>
       </c>
@@ -8353,7 +8358,7 @@
       </c>
       <c r="P88" s="49"/>
     </row>
-    <row r="89" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B89" s="46">
         <v>79</v>
       </c>
@@ -8384,7 +8389,7 @@
       </c>
       <c r="P89" s="49"/>
     </row>
-    <row r="90" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B90" s="46">
         <v>80</v>
       </c>
@@ -8415,7 +8420,7 @@
       </c>
       <c r="P90" s="49"/>
     </row>
-    <row r="91" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B91" s="46">
         <v>81</v>
       </c>
@@ -8446,7 +8451,7 @@
       </c>
       <c r="P91" s="49"/>
     </row>
-    <row r="92" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B92" s="46">
         <v>82</v>
       </c>
@@ -8477,7 +8482,7 @@
       </c>
       <c r="P92" s="49"/>
     </row>
-    <row r="93" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B93" s="46">
         <v>83</v>
       </c>
@@ -8508,7 +8513,7 @@
       </c>
       <c r="P93" s="49"/>
     </row>
-    <row r="94" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B94" s="46">
         <v>84</v>
       </c>
@@ -8539,7 +8544,7 @@
       </c>
       <c r="P94" s="49"/>
     </row>
-    <row r="95" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B95" s="46">
         <v>85</v>
       </c>
@@ -8570,7 +8575,7 @@
       </c>
       <c r="P95" s="49"/>
     </row>
-    <row r="96" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B96" s="46">
         <v>86</v>
       </c>
@@ -8601,7 +8606,7 @@
       </c>
       <c r="P96" s="49"/>
     </row>
-    <row r="97" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B97" s="46">
         <v>87</v>
       </c>
@@ -8632,7 +8637,7 @@
       </c>
       <c r="P97" s="49"/>
     </row>
-    <row r="98" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B98" s="46">
         <v>88</v>
       </c>
@@ -8663,7 +8668,7 @@
       </c>
       <c r="P98" s="49"/>
     </row>
-    <row r="99" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B99" s="46">
         <v>89</v>
       </c>
@@ -8694,7 +8699,7 @@
       </c>
       <c r="P99" s="49"/>
     </row>
-    <row r="100" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B100" s="46">
         <v>90</v>
       </c>
@@ -8725,7 +8730,7 @@
       </c>
       <c r="P100" s="49"/>
     </row>
-    <row r="101" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B101" s="46">
         <v>91</v>
       </c>
@@ -8756,7 +8761,7 @@
       </c>
       <c r="P101" s="49"/>
     </row>
-    <row r="102" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B102" s="46">
         <v>92</v>
       </c>
@@ -8787,7 +8792,7 @@
       </c>
       <c r="P102" s="49"/>
     </row>
-    <row r="103" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B103" s="46">
         <v>93</v>
       </c>
@@ -8818,7 +8823,7 @@
       </c>
       <c r="P103" s="49"/>
     </row>
-    <row r="104" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B104" s="46">
         <v>94</v>
       </c>
@@ -8849,7 +8854,7 @@
       </c>
       <c r="P104" s="49"/>
     </row>
-    <row r="105" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B105" s="46">
         <v>95</v>
       </c>
@@ -8880,7 +8885,7 @@
       </c>
       <c r="P105" s="49"/>
     </row>
-    <row r="106" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B106" s="46">
         <v>96</v>
       </c>
@@ -8911,7 +8916,7 @@
       </c>
       <c r="P106" s="49"/>
     </row>
-    <row r="107" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B107" s="46">
         <v>97</v>
       </c>
@@ -8942,7 +8947,7 @@
       </c>
       <c r="P107" s="49"/>
     </row>
-    <row r="108" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B108" s="46">
         <v>98</v>
       </c>
@@ -8973,7 +8978,7 @@
       </c>
       <c r="P108" s="49"/>
     </row>
-    <row r="109" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B109" s="46">
         <v>99</v>
       </c>
@@ -9004,7 +9009,7 @@
       </c>
       <c r="P109" s="49"/>
     </row>
-    <row r="110" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B110" s="46">
         <v>100</v>
       </c>
@@ -9124,13 +9129,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28A2F053-EB65-4682-A8B4-EF605DDDBF14}">
   <dimension ref="B2:P110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="15" width="18.87890625" customWidth="1"/>
-    <col min="16" max="16" width="64.5859375" customWidth="1"/>
+    <col min="3" max="15" width="18.88671875" customWidth="1"/>
+    <col min="16" max="16" width="64.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C2" s="55" t="s">
         <v>15</v>
       </c>
@@ -9148,7 +9153,7 @@
       <c r="O2" s="55"/>
       <c r="P2" s="55"/>
     </row>
-    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C4" s="53" t="s">
         <v>90</v>
       </c>
@@ -9166,7 +9171,7 @@
       <c r="O4" s="53"/>
       <c r="P4" s="53"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -9182,7 +9187,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C6" s="62" t="s">
         <v>83</v>
       </c>
@@ -9205,7 +9210,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C7" s="62"/>
       <c r="D7" s="13" t="s">
         <v>85</v>
@@ -9216,7 +9221,7 @@
       </c>
       <c r="J7" s="40"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -9239,7 +9244,7 @@
       <c r="O9" s="63"/>
       <c r="P9" s="9"/>
     </row>
-    <row r="10" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="10" t="s">
         <v>81</v>
       </c>
@@ -9286,7 +9291,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="46">
         <v>1</v>
       </c>
@@ -9317,7 +9322,7 @@
       </c>
       <c r="P11" s="49"/>
     </row>
-    <row r="12" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="46">
         <v>2</v>
       </c>
@@ -9348,7 +9353,7 @@
       </c>
       <c r="P12" s="49"/>
     </row>
-    <row r="13" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="46">
         <v>3</v>
       </c>
@@ -9379,7 +9384,7 @@
       </c>
       <c r="P13" s="49"/>
     </row>
-    <row r="14" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="46">
         <v>4</v>
       </c>
@@ -9410,7 +9415,7 @@
       </c>
       <c r="P14" s="49"/>
     </row>
-    <row r="15" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="46">
         <v>5</v>
       </c>
@@ -9441,7 +9446,7 @@
       </c>
       <c r="P15" s="49"/>
     </row>
-    <row r="16" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="46">
         <v>6</v>
       </c>
@@ -9472,7 +9477,7 @@
       </c>
       <c r="P16" s="49"/>
     </row>
-    <row r="17" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="46">
         <v>7</v>
       </c>
@@ -9503,7 +9508,7 @@
       </c>
       <c r="P17" s="49"/>
     </row>
-    <row r="18" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="46">
         <v>8</v>
       </c>
@@ -9534,7 +9539,7 @@
       </c>
       <c r="P18" s="49"/>
     </row>
-    <row r="19" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="46">
         <v>9</v>
       </c>
@@ -9565,7 +9570,7 @@
       </c>
       <c r="P19" s="49"/>
     </row>
-    <row r="20" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="46">
         <v>10</v>
       </c>
@@ -9596,7 +9601,7 @@
       </c>
       <c r="P20" s="49"/>
     </row>
-    <row r="21" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="46">
         <v>11</v>
       </c>
@@ -9627,7 +9632,7 @@
       </c>
       <c r="P21" s="49"/>
     </row>
-    <row r="22" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="46">
         <v>12</v>
       </c>
@@ -9658,7 +9663,7 @@
       </c>
       <c r="P22" s="49"/>
     </row>
-    <row r="23" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="46">
         <v>13</v>
       </c>
@@ -9689,7 +9694,7 @@
       </c>
       <c r="P23" s="49"/>
     </row>
-    <row r="24" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="46">
         <v>14</v>
       </c>
@@ -9720,7 +9725,7 @@
       </c>
       <c r="P24" s="49"/>
     </row>
-    <row r="25" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="46">
         <v>15</v>
       </c>
@@ -9751,7 +9756,7 @@
       </c>
       <c r="P25" s="49"/>
     </row>
-    <row r="26" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="46">
         <v>16</v>
       </c>
@@ -9782,7 +9787,7 @@
       </c>
       <c r="P26" s="49"/>
     </row>
-    <row r="27" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="46">
         <v>17</v>
       </c>
@@ -9813,7 +9818,7 @@
       </c>
       <c r="P27" s="49"/>
     </row>
-    <row r="28" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="46">
         <v>18</v>
       </c>
@@ -9844,7 +9849,7 @@
       </c>
       <c r="P28" s="49"/>
     </row>
-    <row r="29" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="46">
         <v>19</v>
       </c>
@@ -9875,7 +9880,7 @@
       </c>
       <c r="P29" s="49"/>
     </row>
-    <row r="30" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="46">
         <v>20</v>
       </c>
@@ -9906,7 +9911,7 @@
       </c>
       <c r="P30" s="49"/>
     </row>
-    <row r="31" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="46">
         <v>21</v>
       </c>
@@ -9937,7 +9942,7 @@
       </c>
       <c r="P31" s="49"/>
     </row>
-    <row r="32" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="46">
         <v>22</v>
       </c>
@@ -9968,7 +9973,7 @@
       </c>
       <c r="P32" s="49"/>
     </row>
-    <row r="33" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="46">
         <v>23</v>
       </c>
@@ -9999,7 +10004,7 @@
       </c>
       <c r="P33" s="49"/>
     </row>
-    <row r="34" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="46">
         <v>24</v>
       </c>
@@ -10030,7 +10035,7 @@
       </c>
       <c r="P34" s="49"/>
     </row>
-    <row r="35" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="46">
         <v>25</v>
       </c>
@@ -10061,7 +10066,7 @@
       </c>
       <c r="P35" s="49"/>
     </row>
-    <row r="36" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="46">
         <v>26</v>
       </c>
@@ -10092,7 +10097,7 @@
       </c>
       <c r="P36" s="49"/>
     </row>
-    <row r="37" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="46">
         <v>27</v>
       </c>
@@ -10123,7 +10128,7 @@
       </c>
       <c r="P37" s="49"/>
     </row>
-    <row r="38" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="46">
         <v>28</v>
       </c>
@@ -10154,7 +10159,7 @@
       </c>
       <c r="P38" s="49"/>
     </row>
-    <row r="39" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="46">
         <v>29</v>
       </c>
@@ -10185,7 +10190,7 @@
       </c>
       <c r="P39" s="49"/>
     </row>
-    <row r="40" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="46">
         <v>30</v>
       </c>
@@ -10216,7 +10221,7 @@
       </c>
       <c r="P40" s="49"/>
     </row>
-    <row r="41" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="46">
         <v>31</v>
       </c>
@@ -10247,7 +10252,7 @@
       </c>
       <c r="P41" s="49"/>
     </row>
-    <row r="42" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="46">
         <v>32</v>
       </c>
@@ -10278,7 +10283,7 @@
       </c>
       <c r="P42" s="49"/>
     </row>
-    <row r="43" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="46">
         <v>33</v>
       </c>
@@ -10309,7 +10314,7 @@
       </c>
       <c r="P43" s="49"/>
     </row>
-    <row r="44" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="46">
         <v>34</v>
       </c>
@@ -10340,7 +10345,7 @@
       </c>
       <c r="P44" s="49"/>
     </row>
-    <row r="45" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B45" s="46">
         <v>35</v>
       </c>
@@ -10371,7 +10376,7 @@
       </c>
       <c r="P45" s="49"/>
     </row>
-    <row r="46" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B46" s="46">
         <v>36</v>
       </c>
@@ -10402,7 +10407,7 @@
       </c>
       <c r="P46" s="49"/>
     </row>
-    <row r="47" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="46">
         <v>37</v>
       </c>
@@ -10433,7 +10438,7 @@
       </c>
       <c r="P47" s="49"/>
     </row>
-    <row r="48" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="46">
         <v>38</v>
       </c>
@@ -10464,7 +10469,7 @@
       </c>
       <c r="P48" s="49"/>
     </row>
-    <row r="49" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="46">
         <v>39</v>
       </c>
@@ -10495,7 +10500,7 @@
       </c>
       <c r="P49" s="49"/>
     </row>
-    <row r="50" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="46">
         <v>40</v>
       </c>
@@ -10526,7 +10531,7 @@
       </c>
       <c r="P50" s="49"/>
     </row>
-    <row r="51" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="46">
         <v>41</v>
       </c>
@@ -10557,7 +10562,7 @@
       </c>
       <c r="P51" s="49"/>
     </row>
-    <row r="52" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B52" s="46">
         <v>42</v>
       </c>
@@ -10588,7 +10593,7 @@
       </c>
       <c r="P52" s="49"/>
     </row>
-    <row r="53" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B53" s="46">
         <v>43</v>
       </c>
@@ -10619,7 +10624,7 @@
       </c>
       <c r="P53" s="49"/>
     </row>
-    <row r="54" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="46">
         <v>44</v>
       </c>
@@ -10650,7 +10655,7 @@
       </c>
       <c r="P54" s="49"/>
     </row>
-    <row r="55" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B55" s="46">
         <v>45</v>
       </c>
@@ -10681,7 +10686,7 @@
       </c>
       <c r="P55" s="49"/>
     </row>
-    <row r="56" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B56" s="46">
         <v>46</v>
       </c>
@@ -10712,7 +10717,7 @@
       </c>
       <c r="P56" s="49"/>
     </row>
-    <row r="57" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="46">
         <v>47</v>
       </c>
@@ -10743,7 +10748,7 @@
       </c>
       <c r="P57" s="49"/>
     </row>
-    <row r="58" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B58" s="46">
         <v>48</v>
       </c>
@@ -10774,7 +10779,7 @@
       </c>
       <c r="P58" s="49"/>
     </row>
-    <row r="59" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B59" s="46">
         <v>49</v>
       </c>
@@ -10805,7 +10810,7 @@
       </c>
       <c r="P59" s="49"/>
     </row>
-    <row r="60" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="46">
         <v>50</v>
       </c>
@@ -10836,7 +10841,7 @@
       </c>
       <c r="P60" s="49"/>
     </row>
-    <row r="61" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="46">
         <v>51</v>
       </c>
@@ -10867,7 +10872,7 @@
       </c>
       <c r="P61" s="49"/>
     </row>
-    <row r="62" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="46">
         <v>52</v>
       </c>
@@ -10898,7 +10903,7 @@
       </c>
       <c r="P62" s="49"/>
     </row>
-    <row r="63" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B63" s="46">
         <v>53</v>
       </c>
@@ -10929,7 +10934,7 @@
       </c>
       <c r="P63" s="49"/>
     </row>
-    <row r="64" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B64" s="46">
         <v>54</v>
       </c>
@@ -10960,7 +10965,7 @@
       </c>
       <c r="P64" s="49"/>
     </row>
-    <row r="65" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="46">
         <v>55</v>
       </c>
@@ -10991,7 +10996,7 @@
       </c>
       <c r="P65" s="49"/>
     </row>
-    <row r="66" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B66" s="46">
         <v>56</v>
       </c>
@@ -11022,7 +11027,7 @@
       </c>
       <c r="P66" s="49"/>
     </row>
-    <row r="67" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B67" s="46">
         <v>57</v>
       </c>
@@ -11053,7 +11058,7 @@
       </c>
       <c r="P67" s="49"/>
     </row>
-    <row r="68" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B68" s="46">
         <v>58</v>
       </c>
@@ -11084,7 +11089,7 @@
       </c>
       <c r="P68" s="49"/>
     </row>
-    <row r="69" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B69" s="46">
         <v>59</v>
       </c>
@@ -11115,7 +11120,7 @@
       </c>
       <c r="P69" s="49"/>
     </row>
-    <row r="70" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B70" s="46">
         <v>60</v>
       </c>
@@ -11146,7 +11151,7 @@
       </c>
       <c r="P70" s="49"/>
     </row>
-    <row r="71" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B71" s="46">
         <v>61</v>
       </c>
@@ -11177,7 +11182,7 @@
       </c>
       <c r="P71" s="49"/>
     </row>
-    <row r="72" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B72" s="46">
         <v>62</v>
       </c>
@@ -11208,7 +11213,7 @@
       </c>
       <c r="P72" s="49"/>
     </row>
-    <row r="73" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B73" s="46">
         <v>63</v>
       </c>
@@ -11239,7 +11244,7 @@
       </c>
       <c r="P73" s="49"/>
     </row>
-    <row r="74" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B74" s="46">
         <v>64</v>
       </c>
@@ -11270,7 +11275,7 @@
       </c>
       <c r="P74" s="49"/>
     </row>
-    <row r="75" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B75" s="46">
         <v>65</v>
       </c>
@@ -11301,7 +11306,7 @@
       </c>
       <c r="P75" s="49"/>
     </row>
-    <row r="76" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B76" s="46">
         <v>66</v>
       </c>
@@ -11332,7 +11337,7 @@
       </c>
       <c r="P76" s="49"/>
     </row>
-    <row r="77" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B77" s="46">
         <v>67</v>
       </c>
@@ -11363,7 +11368,7 @@
       </c>
       <c r="P77" s="49"/>
     </row>
-    <row r="78" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B78" s="46">
         <v>68</v>
       </c>
@@ -11394,7 +11399,7 @@
       </c>
       <c r="P78" s="49"/>
     </row>
-    <row r="79" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B79" s="46">
         <v>69</v>
       </c>
@@ -11425,7 +11430,7 @@
       </c>
       <c r="P79" s="49"/>
     </row>
-    <row r="80" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B80" s="46">
         <v>70</v>
       </c>
@@ -11456,7 +11461,7 @@
       </c>
       <c r="P80" s="49"/>
     </row>
-    <row r="81" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B81" s="46">
         <v>71</v>
       </c>
@@ -11487,7 +11492,7 @@
       </c>
       <c r="P81" s="49"/>
     </row>
-    <row r="82" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B82" s="46">
         <v>72</v>
       </c>
@@ -11518,7 +11523,7 @@
       </c>
       <c r="P82" s="49"/>
     </row>
-    <row r="83" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B83" s="46">
         <v>73</v>
       </c>
@@ -11549,7 +11554,7 @@
       </c>
       <c r="P83" s="49"/>
     </row>
-    <row r="84" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B84" s="46">
         <v>74</v>
       </c>
@@ -11580,7 +11585,7 @@
       </c>
       <c r="P84" s="49"/>
     </row>
-    <row r="85" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B85" s="46">
         <v>75</v>
       </c>
@@ -11611,7 +11616,7 @@
       </c>
       <c r="P85" s="49"/>
     </row>
-    <row r="86" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B86" s="46">
         <v>76</v>
       </c>
@@ -11642,7 +11647,7 @@
       </c>
       <c r="P86" s="49"/>
     </row>
-    <row r="87" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B87" s="46">
         <v>77</v>
       </c>
@@ -11673,7 +11678,7 @@
       </c>
       <c r="P87" s="49"/>
     </row>
-    <row r="88" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B88" s="46">
         <v>78</v>
       </c>
@@ -11704,7 +11709,7 @@
       </c>
       <c r="P88" s="49"/>
     </row>
-    <row r="89" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B89" s="46">
         <v>79</v>
       </c>
@@ -11735,7 +11740,7 @@
       </c>
       <c r="P89" s="49"/>
     </row>
-    <row r="90" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B90" s="46">
         <v>80</v>
       </c>
@@ -11766,7 +11771,7 @@
       </c>
       <c r="P90" s="49"/>
     </row>
-    <row r="91" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B91" s="46">
         <v>81</v>
       </c>
@@ -11797,7 +11802,7 @@
       </c>
       <c r="P91" s="49"/>
     </row>
-    <row r="92" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B92" s="46">
         <v>82</v>
       </c>
@@ -11828,7 +11833,7 @@
       </c>
       <c r="P92" s="49"/>
     </row>
-    <row r="93" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B93" s="46">
         <v>83</v>
       </c>
@@ -11859,7 +11864,7 @@
       </c>
       <c r="P93" s="49"/>
     </row>
-    <row r="94" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B94" s="46">
         <v>84</v>
       </c>
@@ -11890,7 +11895,7 @@
       </c>
       <c r="P94" s="49"/>
     </row>
-    <row r="95" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B95" s="46">
         <v>85</v>
       </c>
@@ -11921,7 +11926,7 @@
       </c>
       <c r="P95" s="49"/>
     </row>
-    <row r="96" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B96" s="46">
         <v>86</v>
       </c>
@@ -11952,7 +11957,7 @@
       </c>
       <c r="P96" s="49"/>
     </row>
-    <row r="97" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B97" s="46">
         <v>87</v>
       </c>
@@ -11983,7 +11988,7 @@
       </c>
       <c r="P97" s="49"/>
     </row>
-    <row r="98" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B98" s="46">
         <v>88</v>
       </c>
@@ -12014,7 +12019,7 @@
       </c>
       <c r="P98" s="49"/>
     </row>
-    <row r="99" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B99" s="46">
         <v>89</v>
       </c>
@@ -12045,7 +12050,7 @@
       </c>
       <c r="P99" s="49"/>
     </row>
-    <row r="100" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B100" s="46">
         <v>90</v>
       </c>
@@ -12076,7 +12081,7 @@
       </c>
       <c r="P100" s="49"/>
     </row>
-    <row r="101" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B101" s="46">
         <v>91</v>
       </c>
@@ -12107,7 +12112,7 @@
       </c>
       <c r="P101" s="49"/>
     </row>
-    <row r="102" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B102" s="46">
         <v>92</v>
       </c>
@@ -12138,7 +12143,7 @@
       </c>
       <c r="P102" s="49"/>
     </row>
-    <row r="103" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B103" s="46">
         <v>93</v>
       </c>
@@ -12169,7 +12174,7 @@
       </c>
       <c r="P103" s="49"/>
     </row>
-    <row r="104" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B104" s="46">
         <v>94</v>
       </c>
@@ -12200,7 +12205,7 @@
       </c>
       <c r="P104" s="49"/>
     </row>
-    <row r="105" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B105" s="46">
         <v>95</v>
       </c>
@@ -12231,7 +12236,7 @@
       </c>
       <c r="P105" s="49"/>
     </row>
-    <row r="106" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B106" s="46">
         <v>96</v>
       </c>
@@ -12262,7 +12267,7 @@
       </c>
       <c r="P106" s="49"/>
     </row>
-    <row r="107" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B107" s="46">
         <v>97</v>
       </c>
@@ -12293,7 +12298,7 @@
       </c>
       <c r="P107" s="49"/>
     </row>
-    <row r="108" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B108" s="46">
         <v>98</v>
       </c>
@@ -12324,7 +12329,7 @@
       </c>
       <c r="P108" s="49"/>
     </row>
-    <row r="109" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B109" s="46">
         <v>99</v>
       </c>
@@ -12355,7 +12360,7 @@
       </c>
       <c r="P109" s="49"/>
     </row>
-    <row r="110" spans="2:16" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B110" s="46">
         <v>100</v>
       </c>
@@ -12475,19 +12480,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6230FA8A-EA33-4C76-AA54-C885D607690C}">
   <dimension ref="B2:J39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5859375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.87890625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.29296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.87890625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.1171875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.41015625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5859375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="15.5859375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="55" t="s">
         <v>23</v>
       </c>
@@ -12500,7 +12505,7 @@
       <c r="I2" s="55"/>
       <c r="J2" s="55"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B4" s="53" t="s">
         <v>25</v>
       </c>
@@ -12513,7 +12518,7 @@
       <c r="I4" s="53"/>
       <c r="J4" s="53"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="53"/>
       <c r="C5" s="53"/>
       <c r="D5" s="53"/>
@@ -12524,7 +12529,7 @@
       <c r="I5" s="53"/>
       <c r="J5" s="53"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="53"/>
       <c r="C6" s="53"/>
       <c r="D6" s="53"/>
@@ -12535,7 +12540,7 @@
       <c r="I6" s="53"/>
       <c r="J6" s="53"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
@@ -12546,7 +12551,7 @@
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="27" t="s">
         <v>24</v>
       </c>
@@ -12559,7 +12564,7 @@
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="15" t="str">
         <f>IF(ISBLANK(Identification!E14), "", Identification!E14)</f>
         <v>manbuzmun</v>
@@ -12573,7 +12578,7 @@
       <c r="I9" s="14"/>
       <c r="J9" s="14"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B10" s="15" t="str">
         <f>IF(ISBLANK(Identification!E18), "", Identification!E18)</f>
         <v>juaprifer</v>
@@ -12587,7 +12592,7 @@
       <c r="I10" s="14"/>
       <c r="J10" s="14"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B11" s="15" t="str">
         <f>IF(ISBLANK(Identification!E22), "", Identification!E22)</f>
         <v>manlavcor</v>
@@ -12601,7 +12606,7 @@
       <c r="I11" s="14"/>
       <c r="J11" s="14"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B12" s="15" t="str">
         <f>IF(ISBLANK(Identification!E26), "", Identification!E26)</f>
         <v>manortper1</v>
@@ -12615,7 +12620,7 @@
       <c r="I12" s="14"/>
       <c r="J12" s="14"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B13" s="15" t="str">
         <f>IF(ISBLANK(Identification!E30), "", Identification!E30)</f>
         <v>sanrodper</v>
@@ -12629,7 +12634,7 @@
       <c r="I13" s="14"/>
       <c r="J13" s="14"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B14" s="16" t="s">
         <v>92</v>
       </c>
@@ -12642,7 +12647,7 @@
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B15" s="4"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
@@ -12653,7 +12658,7 @@
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B16" s="28" t="s">
         <v>26</v>
       </c>
@@ -12666,7 +12671,7 @@
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B17" s="17" t="s">
         <v>27</v>
       </c>
@@ -12679,7 +12684,7 @@
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B18" s="17" t="s">
         <v>28</v>
       </c>
@@ -12692,7 +12697,7 @@
       <c r="I18" s="14"/>
       <c r="J18" s="14"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B19" s="18" t="s">
         <v>29</v>
       </c>
@@ -12705,7 +12710,7 @@
       <c r="I19" s="14"/>
       <c r="J19" s="14"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B20" s="4"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
@@ -12716,7 +12721,7 @@
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B21" s="28" t="s">
         <v>69</v>
       </c>
@@ -12729,7 +12734,7 @@
       <c r="I21" s="14"/>
       <c r="J21" s="14"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B22" s="19">
         <v>45658</v>
       </c>
@@ -12742,7 +12747,7 @@
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B23" s="20" t="s">
         <v>70</v>
       </c>
@@ -12755,7 +12760,7 @@
       <c r="I23" s="14"/>
       <c r="J23" s="14"/>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
@@ -12766,7 +12771,7 @@
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>34</v>
       </c>
@@ -12783,7 +12788,7 @@
       <c r="I25" s="31"/>
       <c r="J25" s="32"/>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B26" s="21" t="s">
         <v>41</v>
       </c>
@@ -12806,7 +12811,7 @@
       <c r="I26" s="14"/>
       <c r="J26" s="22"/>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="27" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B27" s="21" t="s">
         <v>35</v>
       </c>
@@ -12833,7 +12838,7 @@
       </c>
       <c r="J27" s="22"/>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B28" s="21" t="s">
         <v>36</v>
       </c>
@@ -12858,7 +12863,7 @@
       <c r="I28" s="14"/>
       <c r="J28" s="22"/>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B29" s="21" t="s">
         <v>37</v>
       </c>
@@ -12885,7 +12890,7 @@
       </c>
       <c r="J29" s="22"/>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B30" s="21" t="s">
         <v>38</v>
       </c>
@@ -12912,7 +12917,7 @@
       </c>
       <c r="J30" s="22"/>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B31" s="23" t="s">
         <v>39</v>
       </c>
@@ -12941,7 +12946,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B32" s="24" t="s">
         <v>71</v>
       </c>
@@ -12958,7 +12963,7 @@
       <c r="I32" s="25"/>
       <c r="J32" s="26"/>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
@@ -12969,7 +12974,7 @@
       <c r="I33" s="14"/>
       <c r="J33" s="14"/>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B34" s="35" t="s">
         <v>75</v>
       </c>
@@ -12984,7 +12989,7 @@
       <c r="I34" s="14"/>
       <c r="J34" s="14"/>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B35" s="23" t="s">
         <v>79</v>
       </c>
@@ -12999,7 +13004,7 @@
       <c r="I35" s="14"/>
       <c r="J35" s="14"/>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B36" s="23" t="s">
         <v>77</v>
       </c>
@@ -13014,7 +13019,7 @@
       <c r="I36" s="14"/>
       <c r="J36" s="14"/>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B37" s="23" t="s">
         <v>80</v>
       </c>
@@ -13029,7 +13034,7 @@
       <c r="I37" s="14"/>
       <c r="J37" s="14"/>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B38" s="23" t="s">
         <v>76</v>
       </c>
@@ -13044,7 +13049,7 @@
       <c r="I38" s="14"/>
       <c r="J38" s="14"/>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B39" s="34" t="s">
         <v>71</v>
       </c>

</xml_diff>